<commit_message>
Gafas de sol: 10 variantes finales (SKU, remisión, Siigo y video actualizados)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Nmsujw5inBeAZKWmtCeCB5
</commit_message>
<xml_diff>
--- a/productos/ModeloPersonalizado-ImportacionProductos-20261010114257114-e63b191eb0784ae6b77169edc57c1987.xlsx
+++ b/productos/ModeloPersonalizado-ImportacionProductos-20261010114257114-e63b191eb0784ae6b77169edc57c1987.xlsx
@@ -377,35 +377,6 @@
         <x:v>Hello Mellow</x:v>
       </x:c>
       <x:c t="str">
-        <x:v>HM-GAF-AZR</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>Gafas de sol para niños - Azul rey</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>SI</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>2001001000011</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>1-IVA 19%</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>SI</x:v>
-      </x:c>
-      <x:c>
-        <x:v>29900</x:v>
-      </x:c>
-    </x:row>
-    <x:row>
-      <x:c t="str">
-        <x:v>P-Producto</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>Hello Mellow</x:v>
-      </x:c>
-      <x:c t="str">
         <x:v>HM-GAF-AZC</x:v>
       </x:c>
       <x:c t="str">
@@ -641,71 +612,13 @@
         <x:v>HM-GAF-RN1</x:v>
       </x:c>
       <x:c t="str">
-        <x:v>Gafas de sol para niños - Rayas naranja 1</x:v>
+        <x:v>Gafas de sol para niños - Rayas naranja</x:v>
       </x:c>
       <x:c t="str">
         <x:v>SI</x:v>
       </x:c>
       <x:c t="str">
         <x:v>2001001000103</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>1-IVA 19%</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>SI</x:v>
-      </x:c>
-      <x:c>
-        <x:v>29900</x:v>
-      </x:c>
-    </x:row>
-    <x:row>
-      <x:c t="str">
-        <x:v>P-Producto</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>Hello Mellow</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>HM-GAF-RN2</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>Gafas de sol para niños - Rayas naranja 2</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>SI</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>2001001000110</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>1-IVA 19%</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>SI</x:v>
-      </x:c>
-      <x:c>
-        <x:v>29900</x:v>
-      </x:c>
-    </x:row>
-    <x:row>
-      <x:c t="str">
-        <x:v>P-Producto</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>Hello Mellow</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>HM-GAF-RN3</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>Gafas de sol para niños - Rayas naranja 3</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>SI</x:v>
-      </x:c>
-      <x:c t="str">
-        <x:v>2001001000127</x:v>
       </x:c>
       <x:c t="str">
         <x:v>1-IVA 19%</x:v>

</xml_diff>